<commit_message>
Rebuild CPR FMEA worksheet with cached formula values
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6R5HNSLVTt1JG7dkjH6BA
</commit_message>
<xml_diff>
--- a/CPR_FMEA_워크시트.xlsx
+++ b/CPR_FMEA_워크시트.xlsx
@@ -1127,11 +1127,11 @@
       </c>
       <c r="L5" s="11">
         <f>I5*J5*K5</f>
-        <v/>
-      </c>
-      <c r="M5" s="11">
+        <v>200</v>
+      </c>
+      <c r="M5" s="11" t="str">
         <f>IF(OR(L5&gt;=척도!$B$17,AND(I5&gt;=척도!$B$19,L5&gt;=척도!$B$18)),"높음",IF(L5&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N5" s="12" t="inlineStr">
         <is>
@@ -1194,11 +1194,11 @@
       </c>
       <c r="L6" s="11">
         <f>I6*J6*K6</f>
-        <v/>
-      </c>
-      <c r="M6" s="11">
+        <v>240</v>
+      </c>
+      <c r="M6" s="11" t="str">
         <f>IF(OR(L6&gt;=척도!$B$17,AND(I6&gt;=척도!$B$19,L6&gt;=척도!$B$18)),"높음",IF(L6&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
@@ -1261,11 +1261,11 @@
       </c>
       <c r="L7" s="11">
         <f>I7*J7*K7</f>
-        <v/>
-      </c>
-      <c r="M7" s="11">
+        <v>288</v>
+      </c>
+      <c r="M7" s="11" t="str">
         <f>IF(OR(L7&gt;=척도!$B$17,AND(I7&gt;=척도!$B$19,L7&gt;=척도!$B$18)),"높음",IF(L7&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N7" s="12" t="inlineStr">
         <is>
@@ -1328,11 +1328,11 @@
       </c>
       <c r="L8" s="11">
         <f>I8*J8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="11">
+        <v>280</v>
+      </c>
+      <c r="M8" s="11" t="str">
         <f>IF(OR(L8&gt;=척도!$B$17,AND(I8&gt;=척도!$B$19,L8&gt;=척도!$B$18)),"높음",IF(L8&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
@@ -1395,11 +1395,11 @@
       </c>
       <c r="L9" s="11">
         <f>I9*J9*K9</f>
-        <v/>
-      </c>
-      <c r="M9" s="11">
+        <v>240</v>
+      </c>
+      <c r="M9" s="11" t="str">
         <f>IF(OR(L9&gt;=척도!$B$17,AND(I9&gt;=척도!$B$19,L9&gt;=척도!$B$18)),"높음",IF(L9&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N9" s="12" t="inlineStr">
         <is>
@@ -1462,11 +1462,11 @@
       </c>
       <c r="L10" s="11">
         <f>I10*J10*K10</f>
-        <v/>
-      </c>
-      <c r="M10" s="11">
+        <v>180</v>
+      </c>
+      <c r="M10" s="11" t="str">
         <f>IF(OR(L10&gt;=척도!$B$17,AND(I10&gt;=척도!$B$19,L10&gt;=척도!$B$18)),"높음",IF(L10&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
@@ -1529,11 +1529,11 @@
       </c>
       <c r="L11" s="11">
         <f>I11*J11*K11</f>
-        <v/>
-      </c>
-      <c r="M11" s="11">
+        <v>300</v>
+      </c>
+      <c r="M11" s="11" t="str">
         <f>IF(OR(L11&gt;=척도!$B$17,AND(I11&gt;=척도!$B$19,L11&gt;=척도!$B$18)),"높음",IF(L11&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
@@ -1596,11 +1596,11 @@
       </c>
       <c r="L12" s="11">
         <f>I12*J12*K12</f>
-        <v/>
-      </c>
-      <c r="M12" s="11">
+        <v>270</v>
+      </c>
+      <c r="M12" s="11" t="str">
         <f>IF(OR(L12&gt;=척도!$B$17,AND(I12&gt;=척도!$B$19,L12&gt;=척도!$B$18)),"높음",IF(L12&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
@@ -1663,11 +1663,11 @@
       </c>
       <c r="L13" s="11">
         <f>I13*J13*K13</f>
-        <v/>
-      </c>
-      <c r="M13" s="11">
+        <v>270</v>
+      </c>
+      <c r="M13" s="11" t="str">
         <f>IF(OR(L13&gt;=척도!$B$17,AND(I13&gt;=척도!$B$19,L13&gt;=척도!$B$18)),"높음",IF(L13&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N13" s="12" t="inlineStr">
         <is>
@@ -1730,11 +1730,11 @@
       </c>
       <c r="L14" s="11">
         <f>I14*J14*K14</f>
-        <v/>
-      </c>
-      <c r="M14" s="11">
+        <v>216</v>
+      </c>
+      <c r="M14" s="11" t="str">
         <f>IF(OR(L14&gt;=척도!$B$17,AND(I14&gt;=척도!$B$19,L14&gt;=척도!$B$18)),"높음",IF(L14&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N14" s="12" t="inlineStr">
         <is>
@@ -1797,11 +1797,11 @@
       </c>
       <c r="L15" s="11">
         <f>I15*J15*K15</f>
-        <v/>
-      </c>
-      <c r="M15" s="11">
+        <v>250</v>
+      </c>
+      <c r="M15" s="11" t="str">
         <f>IF(OR(L15&gt;=척도!$B$17,AND(I15&gt;=척도!$B$19,L15&gt;=척도!$B$18)),"높음",IF(L15&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
@@ -1864,11 +1864,11 @@
       </c>
       <c r="L16" s="11">
         <f>I16*J16*K16</f>
-        <v/>
-      </c>
-      <c r="M16" s="11">
+        <v>180</v>
+      </c>
+      <c r="M16" s="11" t="str">
         <f>IF(OR(L16&gt;=척도!$B$17,AND(I16&gt;=척도!$B$19,L16&gt;=척도!$B$18)),"높음",IF(L16&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N16" s="12" t="inlineStr">
         <is>
@@ -1931,11 +1931,11 @@
       </c>
       <c r="L17" s="11">
         <f>I17*J17*K17</f>
-        <v/>
-      </c>
-      <c r="M17" s="11">
+        <v>270</v>
+      </c>
+      <c r="M17" s="11" t="str">
         <f>IF(OR(L17&gt;=척도!$B$17,AND(I17&gt;=척도!$B$19,L17&gt;=척도!$B$18)),"높음",IF(L17&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N17" s="12" t="inlineStr">
         <is>
@@ -1998,11 +1998,11 @@
       </c>
       <c r="L18" s="11">
         <f>I18*J18*K18</f>
-        <v/>
-      </c>
-      <c r="M18" s="11">
+        <v>175</v>
+      </c>
+      <c r="M18" s="11" t="str">
         <f>IF(OR(L18&gt;=척도!$B$17,AND(I18&gt;=척도!$B$19,L18&gt;=척도!$B$18)),"높음",IF(L18&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
@@ -2065,11 +2065,11 @@
       </c>
       <c r="L19" s="11">
         <f>I19*J19*K19</f>
-        <v/>
-      </c>
-      <c r="M19" s="11">
+        <v>225</v>
+      </c>
+      <c r="M19" s="11" t="str">
         <f>IF(OR(L19&gt;=척도!$B$17,AND(I19&gt;=척도!$B$19,L19&gt;=척도!$B$18)),"높음",IF(L19&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
@@ -2132,11 +2132,11 @@
       </c>
       <c r="L20" s="11">
         <f>I20*J20*K20</f>
-        <v/>
-      </c>
-      <c r="M20" s="11">
+        <v>240</v>
+      </c>
+      <c r="M20" s="11" t="str">
         <f>IF(OR(L20&gt;=척도!$B$17,AND(I20&gt;=척도!$B$19,L20&gt;=척도!$B$18)),"높음",IF(L20&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
@@ -2199,11 +2199,11 @@
       </c>
       <c r="L21" s="11">
         <f>I21*J21*K21</f>
-        <v/>
-      </c>
-      <c r="M21" s="11">
+        <v>250</v>
+      </c>
+      <c r="M21" s="11" t="str">
         <f>IF(OR(L21&gt;=척도!$B$17,AND(I21&gt;=척도!$B$19,L21&gt;=척도!$B$18)),"높음",IF(L21&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
@@ -2266,11 +2266,11 @@
       </c>
       <c r="L22" s="11">
         <f>I22*J22*K22</f>
-        <v/>
-      </c>
-      <c r="M22" s="11">
+        <v>378</v>
+      </c>
+      <c r="M22" s="11" t="str">
         <f>IF(OR(L22&gt;=척도!$B$17,AND(I22&gt;=척도!$B$19,L22&gt;=척도!$B$18)),"높음",IF(L22&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N22" s="12" t="inlineStr">
         <is>
@@ -2333,11 +2333,11 @@
       </c>
       <c r="L23" s="11">
         <f>I23*J23*K23</f>
-        <v/>
-      </c>
-      <c r="M23" s="11">
+        <v>378</v>
+      </c>
+      <c r="M23" s="11" t="str">
         <f>IF(OR(L23&gt;=척도!$B$17,AND(I23&gt;=척도!$B$19,L23&gt;=척도!$B$18)),"높음",IF(L23&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N23" s="12" t="inlineStr">
         <is>
@@ -2400,11 +2400,11 @@
       </c>
       <c r="L24" s="11">
         <f>I24*J24*K24</f>
-        <v/>
-      </c>
-      <c r="M24" s="11">
+        <v>288</v>
+      </c>
+      <c r="M24" s="11" t="str">
         <f>IF(OR(L24&gt;=척도!$B$17,AND(I24&gt;=척도!$B$19,L24&gt;=척도!$B$18)),"높음",IF(L24&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N24" s="12" t="inlineStr">
         <is>
@@ -2467,11 +2467,11 @@
       </c>
       <c r="L25" s="11">
         <f>I25*J25*K25</f>
-        <v/>
-      </c>
-      <c r="M25" s="11">
+        <v>245</v>
+      </c>
+      <c r="M25" s="11" t="str">
         <f>IF(OR(L25&gt;=척도!$B$17,AND(I25&gt;=척도!$B$19,L25&gt;=척도!$B$18)),"높음",IF(L25&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N25" s="12" t="inlineStr">
         <is>
@@ -2534,11 +2534,11 @@
       </c>
       <c r="L26" s="11">
         <f>I26*J26*K26</f>
-        <v/>
-      </c>
-      <c r="M26" s="11">
+        <v>225</v>
+      </c>
+      <c r="M26" s="11" t="str">
         <f>IF(OR(L26&gt;=척도!$B$17,AND(I26&gt;=척도!$B$19,L26&gt;=척도!$B$18)),"높음",IF(L26&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
@@ -2601,11 +2601,11 @@
       </c>
       <c r="L27" s="11">
         <f>I27*J27*K27</f>
-        <v/>
-      </c>
-      <c r="M27" s="11">
+        <v>180</v>
+      </c>
+      <c r="M27" s="11" t="str">
         <f>IF(OR(L27&gt;=척도!$B$17,AND(I27&gt;=척도!$B$19,L27&gt;=척도!$B$18)),"높음",IF(L27&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N27" s="12" t="inlineStr">
         <is>
@@ -2668,11 +2668,11 @@
       </c>
       <c r="L28" s="11">
         <f>I28*J28*K28</f>
-        <v/>
-      </c>
-      <c r="M28" s="11">
+        <v>250</v>
+      </c>
+      <c r="M28" s="11" t="str">
         <f>IF(OR(L28&gt;=척도!$B$17,AND(I28&gt;=척도!$B$19,L28&gt;=척도!$B$18)),"높음",IF(L28&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N28" s="12" t="inlineStr">
         <is>
@@ -2735,11 +2735,11 @@
       </c>
       <c r="L29" s="11">
         <f>I29*J29*K29</f>
-        <v/>
-      </c>
-      <c r="M29" s="11">
+        <v>240</v>
+      </c>
+      <c r="M29" s="11" t="str">
         <f>IF(OR(L29&gt;=척도!$B$17,AND(I29&gt;=척도!$B$19,L29&gt;=척도!$B$18)),"높음",IF(L29&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N29" s="12" t="inlineStr">
         <is>
@@ -2802,11 +2802,11 @@
       </c>
       <c r="L30" s="11">
         <f>I30*J30*K30</f>
-        <v/>
-      </c>
-      <c r="M30" s="11">
+        <v>200</v>
+      </c>
+      <c r="M30" s="11" t="str">
         <f>IF(OR(L30&gt;=척도!$B$17,AND(I30&gt;=척도!$B$19,L30&gt;=척도!$B$18)),"높음",IF(L30&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N30" s="12" t="inlineStr">
         <is>
@@ -2869,11 +2869,11 @@
       </c>
       <c r="L31" s="11">
         <f>I31*J31*K31</f>
-        <v/>
-      </c>
-      <c r="M31" s="11">
+        <v>270</v>
+      </c>
+      <c r="M31" s="11" t="str">
         <f>IF(OR(L31&gt;=척도!$B$17,AND(I31&gt;=척도!$B$19,L31&gt;=척도!$B$18)),"높음",IF(L31&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N31" s="12" t="inlineStr">
         <is>
@@ -2936,11 +2936,11 @@
       </c>
       <c r="L32" s="11">
         <f>I32*J32*K32</f>
-        <v/>
-      </c>
-      <c r="M32" s="11">
+        <v>288</v>
+      </c>
+      <c r="M32" s="11" t="str">
         <f>IF(OR(L32&gt;=척도!$B$17,AND(I32&gt;=척도!$B$19,L32&gt;=척도!$B$18)),"높음",IF(L32&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N32" s="12" t="inlineStr">
         <is>
@@ -3003,11 +3003,11 @@
       </c>
       <c r="L33" s="11">
         <f>I33*J33*K33</f>
-        <v/>
-      </c>
-      <c r="M33" s="11">
+        <v>270</v>
+      </c>
+      <c r="M33" s="11" t="str">
         <f>IF(OR(L33&gt;=척도!$B$17,AND(I33&gt;=척도!$B$19,L33&gt;=척도!$B$18)),"높음",IF(L33&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N33" s="12" t="inlineStr">
         <is>
@@ -3070,11 +3070,11 @@
       </c>
       <c r="L34" s="11">
         <f>I34*J34*K34</f>
-        <v/>
-      </c>
-      <c r="M34" s="11">
+        <v>250</v>
+      </c>
+      <c r="M34" s="11" t="str">
         <f>IF(OR(L34&gt;=척도!$B$17,AND(I34&gt;=척도!$B$19,L34&gt;=척도!$B$18)),"높음",IF(L34&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N34" s="12" t="inlineStr">
         <is>
@@ -3137,11 +3137,11 @@
       </c>
       <c r="L35" s="11">
         <f>I35*J35*K35</f>
-        <v/>
-      </c>
-      <c r="M35" s="11">
+        <v>180</v>
+      </c>
+      <c r="M35" s="11" t="str">
         <f>IF(OR(L35&gt;=척도!$B$17,AND(I35&gt;=척도!$B$19,L35&gt;=척도!$B$18)),"높음",IF(L35&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N35" s="12" t="inlineStr">
         <is>
@@ -3204,11 +3204,11 @@
       </c>
       <c r="L36" s="11">
         <f>I36*J36*K36</f>
-        <v/>
-      </c>
-      <c r="M36" s="11">
+        <v>240</v>
+      </c>
+      <c r="M36" s="11" t="str">
         <f>IF(OR(L36&gt;=척도!$B$17,AND(I36&gt;=척도!$B$19,L36&gt;=척도!$B$18)),"높음",IF(L36&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N36" s="12" t="inlineStr">
         <is>
@@ -3271,11 +3271,11 @@
       </c>
       <c r="L37" s="11">
         <f>I37*J37*K37</f>
-        <v/>
-      </c>
-      <c r="M37" s="11">
+        <v>270</v>
+      </c>
+      <c r="M37" s="11" t="str">
         <f>IF(OR(L37&gt;=척도!$B$17,AND(I37&gt;=척도!$B$19,L37&gt;=척도!$B$18)),"높음",IF(L37&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N37" s="12" t="inlineStr">
         <is>
@@ -3338,11 +3338,11 @@
       </c>
       <c r="L38" s="11">
         <f>I38*J38*K38</f>
-        <v/>
-      </c>
-      <c r="M38" s="11">
+        <v>240</v>
+      </c>
+      <c r="M38" s="11" t="str">
         <f>IF(OR(L38&gt;=척도!$B$17,AND(I38&gt;=척도!$B$19,L38&gt;=척도!$B$18)),"높음",IF(L38&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
@@ -3405,11 +3405,11 @@
       </c>
       <c r="L39" s="11">
         <f>I39*J39*K39</f>
-        <v/>
-      </c>
-      <c r="M39" s="11">
+        <v>210</v>
+      </c>
+      <c r="M39" s="11" t="str">
         <f>IF(OR(L39&gt;=척도!$B$17,AND(I39&gt;=척도!$B$19,L39&gt;=척도!$B$18)),"높음",IF(L39&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N39" s="12" t="inlineStr">
         <is>
@@ -3472,11 +3472,11 @@
       </c>
       <c r="L40" s="11">
         <f>I40*J40*K40</f>
-        <v/>
-      </c>
-      <c r="M40" s="11">
+        <v>250</v>
+      </c>
+      <c r="M40" s="11" t="str">
         <f>IF(OR(L40&gt;=척도!$B$17,AND(I40&gt;=척도!$B$19,L40&gt;=척도!$B$18)),"높음",IF(L40&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
@@ -3539,11 +3539,11 @@
       </c>
       <c r="L41" s="11">
         <f>I41*J41*K41</f>
-        <v/>
-      </c>
-      <c r="M41" s="11">
+        <v>240</v>
+      </c>
+      <c r="M41" s="11" t="str">
         <f>IF(OR(L41&gt;=척도!$B$17,AND(I41&gt;=척도!$B$19,L41&gt;=척도!$B$18)),"높음",IF(L41&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N41" s="12" t="inlineStr">
         <is>
@@ -3606,11 +3606,11 @@
       </c>
       <c r="L42" s="11">
         <f>I42*J42*K42</f>
-        <v/>
-      </c>
-      <c r="M42" s="11">
+        <v>378</v>
+      </c>
+      <c r="M42" s="11" t="str">
         <f>IF(OR(L42&gt;=척도!$B$17,AND(I42&gt;=척도!$B$19,L42&gt;=척도!$B$18)),"높음",IF(L42&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
@@ -3673,11 +3673,11 @@
       </c>
       <c r="L43" s="11">
         <f>I43*J43*K43</f>
-        <v/>
-      </c>
-      <c r="M43" s="11">
+        <v>252</v>
+      </c>
+      <c r="M43" s="11" t="str">
         <f>IF(OR(L43&gt;=척도!$B$17,AND(I43&gt;=척도!$B$19,L43&gt;=척도!$B$18)),"높음",IF(L43&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N43" s="12" t="inlineStr">
         <is>
@@ -3740,11 +3740,11 @@
       </c>
       <c r="L44" s="11">
         <f>I44*J44*K44</f>
-        <v/>
-      </c>
-      <c r="M44" s="11">
+        <v>225</v>
+      </c>
+      <c r="M44" s="11" t="str">
         <f>IF(OR(L44&gt;=척도!$B$17,AND(I44&gt;=척도!$B$19,L44&gt;=척도!$B$18)),"높음",IF(L44&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
@@ -3807,11 +3807,11 @@
       </c>
       <c r="L45" s="11">
         <f>I45*J45*K45</f>
-        <v/>
-      </c>
-      <c r="M45" s="11">
+        <v>210</v>
+      </c>
+      <c r="M45" s="11" t="str">
         <f>IF(OR(L45&gt;=척도!$B$17,AND(I45&gt;=척도!$B$19,L45&gt;=척도!$B$18)),"높음",IF(L45&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N45" s="12" t="inlineStr">
         <is>
@@ -3874,11 +3874,11 @@
       </c>
       <c r="L46" s="11">
         <f>I46*J46*K46</f>
-        <v/>
-      </c>
-      <c r="M46" s="11">
+        <v>240</v>
+      </c>
+      <c r="M46" s="11" t="str">
         <f>IF(OR(L46&gt;=척도!$B$17,AND(I46&gt;=척도!$B$19,L46&gt;=척도!$B$18)),"높음",IF(L46&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
@@ -3941,11 +3941,11 @@
       </c>
       <c r="L47" s="11">
         <f>I47*J47*K47</f>
-        <v/>
-      </c>
-      <c r="M47" s="11">
+        <v>200</v>
+      </c>
+      <c r="M47" s="11" t="str">
         <f>IF(OR(L47&gt;=척도!$B$17,AND(I47&gt;=척도!$B$19,L47&gt;=척도!$B$18)),"높음",IF(L47&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N47" s="12" t="inlineStr">
         <is>
@@ -4008,11 +4008,11 @@
       </c>
       <c r="L48" s="11">
         <f>I48*J48*K48</f>
-        <v/>
-      </c>
-      <c r="M48" s="11">
+        <v>270</v>
+      </c>
+      <c r="M48" s="11" t="str">
         <f>IF(OR(L48&gt;=척도!$B$17,AND(I48&gt;=척도!$B$19,L48&gt;=척도!$B$18)),"높음",IF(L48&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
@@ -4075,11 +4075,11 @@
       </c>
       <c r="L49" s="11">
         <f>I49*J49*K49</f>
-        <v/>
-      </c>
-      <c r="M49" s="11">
+        <v>225</v>
+      </c>
+      <c r="M49" s="11" t="str">
         <f>IF(OR(L49&gt;=척도!$B$17,AND(I49&gt;=척도!$B$19,L49&gt;=척도!$B$18)),"높음",IF(L49&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N49" s="12" t="inlineStr">
         <is>
@@ -4142,11 +4142,11 @@
       </c>
       <c r="L50" s="11">
         <f>I50*J50*K50</f>
-        <v/>
-      </c>
-      <c r="M50" s="11">
+        <v>216</v>
+      </c>
+      <c r="M50" s="11" t="str">
         <f>IF(OR(L50&gt;=척도!$B$17,AND(I50&gt;=척도!$B$19,L50&gt;=척도!$B$18)),"높음",IF(L50&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
@@ -4209,11 +4209,11 @@
       </c>
       <c r="L51" s="11">
         <f>I51*J51*K51</f>
-        <v/>
-      </c>
-      <c r="M51" s="11">
+        <v>288</v>
+      </c>
+      <c r="M51" s="11" t="str">
         <f>IF(OR(L51&gt;=척도!$B$17,AND(I51&gt;=척도!$B$19,L51&gt;=척도!$B$18)),"높음",IF(L51&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N51" s="12" t="inlineStr">
         <is>
@@ -4276,11 +4276,11 @@
       </c>
       <c r="L52" s="11">
         <f>I52*J52*K52</f>
-        <v/>
-      </c>
-      <c r="M52" s="11">
+        <v>324</v>
+      </c>
+      <c r="M52" s="11" t="str">
         <f>IF(OR(L52&gt;=척도!$B$17,AND(I52&gt;=척도!$B$19,L52&gt;=척도!$B$18)),"높음",IF(L52&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
@@ -4343,11 +4343,11 @@
       </c>
       <c r="L53" s="11">
         <f>I53*J53*K53</f>
-        <v/>
-      </c>
-      <c r="M53" s="11">
+        <v>252</v>
+      </c>
+      <c r="M53" s="11" t="str">
         <f>IF(OR(L53&gt;=척도!$B$17,AND(I53&gt;=척도!$B$19,L53&gt;=척도!$B$18)),"높음",IF(L53&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N53" s="12" t="inlineStr">
         <is>
@@ -4410,11 +4410,11 @@
       </c>
       <c r="L54" s="11">
         <f>I54*J54*K54</f>
-        <v/>
-      </c>
-      <c r="M54" s="11">
+        <v>180</v>
+      </c>
+      <c r="M54" s="11" t="str">
         <f>IF(OR(L54&gt;=척도!$B$17,AND(I54&gt;=척도!$B$19,L54&gt;=척도!$B$18)),"높음",IF(L54&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
@@ -4477,11 +4477,11 @@
       </c>
       <c r="L55" s="11">
         <f>I55*J55*K55</f>
-        <v/>
-      </c>
-      <c r="M55" s="11">
+        <v>180</v>
+      </c>
+      <c r="M55" s="11" t="str">
         <f>IF(OR(L55&gt;=척도!$B$17,AND(I55&gt;=척도!$B$19,L55&gt;=척도!$B$18)),"높음",IF(L55&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N55" s="12" t="inlineStr">
         <is>
@@ -4544,11 +4544,11 @@
       </c>
       <c r="L56" s="11">
         <f>I56*J56*K56</f>
-        <v/>
-      </c>
-      <c r="M56" s="11">
+        <v>324</v>
+      </c>
+      <c r="M56" s="11" t="str">
         <f>IF(OR(L56&gt;=척도!$B$17,AND(I56&gt;=척도!$B$19,L56&gt;=척도!$B$18)),"높음",IF(L56&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
@@ -4611,11 +4611,11 @@
       </c>
       <c r="L57" s="11">
         <f>I57*J57*K57</f>
-        <v/>
-      </c>
-      <c r="M57" s="11">
+        <v>270</v>
+      </c>
+      <c r="M57" s="11" t="str">
         <f>IF(OR(L57&gt;=척도!$B$17,AND(I57&gt;=척도!$B$19,L57&gt;=척도!$B$18)),"높음",IF(L57&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N57" s="12" t="inlineStr">
         <is>
@@ -4678,11 +4678,11 @@
       </c>
       <c r="L58" s="11">
         <f>I58*J58*K58</f>
-        <v/>
-      </c>
-      <c r="M58" s="11">
+        <v>288</v>
+      </c>
+      <c r="M58" s="11" t="str">
         <f>IF(OR(L58&gt;=척도!$B$17,AND(I58&gt;=척도!$B$19,L58&gt;=척도!$B$18)),"높음",IF(L58&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
@@ -4745,11 +4745,11 @@
       </c>
       <c r="L59" s="11">
         <f>I59*J59*K59</f>
-        <v/>
-      </c>
-      <c r="M59" s="11">
+        <v>240</v>
+      </c>
+      <c r="M59" s="11" t="str">
         <f>IF(OR(L59&gt;=척도!$B$17,AND(I59&gt;=척도!$B$19,L59&gt;=척도!$B$18)),"높음",IF(L59&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N59" s="12" t="inlineStr">
         <is>
@@ -4812,11 +4812,11 @@
       </c>
       <c r="L60" s="11">
         <f>I60*J60*K60</f>
-        <v/>
-      </c>
-      <c r="M60" s="11">
+        <v>270</v>
+      </c>
+      <c r="M60" s="11" t="str">
         <f>IF(OR(L60&gt;=척도!$B$17,AND(I60&gt;=척도!$B$19,L60&gt;=척도!$B$18)),"높음",IF(L60&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
@@ -4879,11 +4879,11 @@
       </c>
       <c r="L61" s="11">
         <f>I61*J61*K61</f>
-        <v/>
-      </c>
-      <c r="M61" s="11">
+        <v>240</v>
+      </c>
+      <c r="M61" s="11" t="str">
         <f>IF(OR(L61&gt;=척도!$B$17,AND(I61&gt;=척도!$B$19,L61&gt;=척도!$B$18)),"높음",IF(L61&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N61" s="12" t="inlineStr">
         <is>
@@ -4946,11 +4946,11 @@
       </c>
       <c r="L62" s="11">
         <f>I62*J62*K62</f>
-        <v/>
-      </c>
-      <c r="M62" s="11">
+        <v>336</v>
+      </c>
+      <c r="M62" s="11" t="str">
         <f>IF(OR(L62&gt;=척도!$B$17,AND(I62&gt;=척도!$B$19,L62&gt;=척도!$B$18)),"높음",IF(L62&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N62" s="12" t="inlineStr">
         <is>
@@ -5013,11 +5013,11 @@
       </c>
       <c r="L63" s="11">
         <f>I63*J63*K63</f>
-        <v/>
-      </c>
-      <c r="M63" s="11">
+        <v>343</v>
+      </c>
+      <c r="M63" s="11" t="str">
         <f>IF(OR(L63&gt;=척도!$B$17,AND(I63&gt;=척도!$B$19,L63&gt;=척도!$B$18)),"높음",IF(L63&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N63" s="12" t="inlineStr">
         <is>
@@ -5232,11 +5232,11 @@
       </c>
       <c r="L5" s="11">
         <f>I5*J5*K5</f>
-        <v/>
-      </c>
-      <c r="M5" s="11">
+        <v>288</v>
+      </c>
+      <c r="M5" s="11" t="str">
         <f>IF(OR(L5&gt;=척도!$B$17,AND(I5&gt;=척도!$B$19,L5&gt;=척도!$B$18)),"높음",IF(L5&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N5" s="12" t="inlineStr">
         <is>
@@ -5299,11 +5299,11 @@
       </c>
       <c r="L6" s="11">
         <f>I6*J6*K6</f>
-        <v/>
-      </c>
-      <c r="M6" s="11">
+        <v>294</v>
+      </c>
+      <c r="M6" s="11" t="str">
         <f>IF(OR(L6&gt;=척도!$B$17,AND(I6&gt;=척도!$B$19,L6&gt;=척도!$B$18)),"높음",IF(L6&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
@@ -5366,11 +5366,11 @@
       </c>
       <c r="L7" s="11">
         <f>I7*J7*K7</f>
-        <v/>
-      </c>
-      <c r="M7" s="11">
+        <v>270</v>
+      </c>
+      <c r="M7" s="11" t="str">
         <f>IF(OR(L7&gt;=척도!$B$17,AND(I7&gt;=척도!$B$19,L7&gt;=척도!$B$18)),"높음",IF(L7&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N7" s="12" t="inlineStr">
         <is>
@@ -5433,11 +5433,11 @@
       </c>
       <c r="L8" s="11">
         <f>I8*J8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="11">
+        <v>210</v>
+      </c>
+      <c r="M8" s="11" t="str">
         <f>IF(OR(L8&gt;=척도!$B$17,AND(I8&gt;=척도!$B$19,L8&gt;=척도!$B$18)),"높음",IF(L8&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
@@ -5500,11 +5500,11 @@
       </c>
       <c r="L9" s="11">
         <f>I9*J9*K9</f>
-        <v/>
-      </c>
-      <c r="M9" s="11">
+        <v>441</v>
+      </c>
+      <c r="M9" s="11" t="str">
         <f>IF(OR(L9&gt;=척도!$B$17,AND(I9&gt;=척도!$B$19,L9&gt;=척도!$B$18)),"높음",IF(L9&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N9" s="12" t="inlineStr">
         <is>
@@ -5567,11 +5567,11 @@
       </c>
       <c r="L10" s="11">
         <f>I10*J10*K10</f>
-        <v/>
-      </c>
-      <c r="M10" s="11">
+        <v>245</v>
+      </c>
+      <c r="M10" s="11" t="str">
         <f>IF(OR(L10&gt;=척도!$B$17,AND(I10&gt;=척도!$B$19,L10&gt;=척도!$B$18)),"높음",IF(L10&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
@@ -5634,11 +5634,11 @@
       </c>
       <c r="L11" s="11">
         <f>I11*J11*K11</f>
-        <v/>
-      </c>
-      <c r="M11" s="11">
+        <v>280</v>
+      </c>
+      <c r="M11" s="11" t="str">
         <f>IF(OR(L11&gt;=척도!$B$17,AND(I11&gt;=척도!$B$19,L11&gt;=척도!$B$18)),"높음",IF(L11&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
@@ -5701,11 +5701,11 @@
       </c>
       <c r="L12" s="11">
         <f>I12*J12*K12</f>
-        <v/>
-      </c>
-      <c r="M12" s="11">
+        <v>240</v>
+      </c>
+      <c r="M12" s="11" t="str">
         <f>IF(OR(L12&gt;=척도!$B$17,AND(I12&gt;=척도!$B$19,L12&gt;=척도!$B$18)),"높음",IF(L12&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
@@ -5768,11 +5768,11 @@
       </c>
       <c r="L13" s="11">
         <f>I13*J13*K13</f>
-        <v/>
-      </c>
-      <c r="M13" s="11">
+        <v>288</v>
+      </c>
+      <c r="M13" s="11" t="str">
         <f>IF(OR(L13&gt;=척도!$B$17,AND(I13&gt;=척도!$B$19,L13&gt;=척도!$B$18)),"높음",IF(L13&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N13" s="12" t="inlineStr">
         <is>
@@ -5835,11 +5835,11 @@
       </c>
       <c r="L14" s="11">
         <f>I14*J14*K14</f>
-        <v/>
-      </c>
-      <c r="M14" s="11">
+        <v>350</v>
+      </c>
+      <c r="M14" s="11" t="str">
         <f>IF(OR(L14&gt;=척도!$B$17,AND(I14&gt;=척도!$B$19,L14&gt;=척도!$B$18)),"높음",IF(L14&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N14" s="12" t="inlineStr">
         <is>
@@ -5902,11 +5902,11 @@
       </c>
       <c r="L15" s="11">
         <f>I15*J15*K15</f>
-        <v/>
-      </c>
-      <c r="M15" s="11">
+        <v>378</v>
+      </c>
+      <c r="M15" s="11" t="str">
         <f>IF(OR(L15&gt;=척도!$B$17,AND(I15&gt;=척도!$B$19,L15&gt;=척도!$B$18)),"높음",IF(L15&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
@@ -5969,11 +5969,11 @@
       </c>
       <c r="L16" s="11">
         <f>I16*J16*K16</f>
-        <v/>
-      </c>
-      <c r="M16" s="11">
+        <v>315</v>
+      </c>
+      <c r="M16" s="11" t="str">
         <f>IF(OR(L16&gt;=척도!$B$17,AND(I16&gt;=척도!$B$19,L16&gt;=척도!$B$18)),"높음",IF(L16&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N16" s="12" t="inlineStr">
         <is>
@@ -6036,11 +6036,11 @@
       </c>
       <c r="L17" s="11">
         <f>I17*J17*K17</f>
-        <v/>
-      </c>
-      <c r="M17" s="11">
+        <v>315</v>
+      </c>
+      <c r="M17" s="11" t="str">
         <f>IF(OR(L17&gt;=척도!$B$17,AND(I17&gt;=척도!$B$19,L17&gt;=척도!$B$18)),"높음",IF(L17&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N17" s="12" t="inlineStr">
         <is>
@@ -6103,11 +6103,11 @@
       </c>
       <c r="L18" s="11">
         <f>I18*J18*K18</f>
-        <v/>
-      </c>
-      <c r="M18" s="11">
+        <v>294</v>
+      </c>
+      <c r="M18" s="11" t="str">
         <f>IF(OR(L18&gt;=척도!$B$17,AND(I18&gt;=척도!$B$19,L18&gt;=척도!$B$18)),"높음",IF(L18&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
@@ -6170,11 +6170,11 @@
       </c>
       <c r="L19" s="11">
         <f>I19*J19*K19</f>
-        <v/>
-      </c>
-      <c r="M19" s="11">
+        <v>294</v>
+      </c>
+      <c r="M19" s="11" t="str">
         <f>IF(OR(L19&gt;=척도!$B$17,AND(I19&gt;=척도!$B$19,L19&gt;=척도!$B$18)),"높음",IF(L19&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
@@ -6237,11 +6237,11 @@
       </c>
       <c r="L20" s="11">
         <f>I20*J20*K20</f>
-        <v/>
-      </c>
-      <c r="M20" s="11">
+        <v>378</v>
+      </c>
+      <c r="M20" s="11" t="str">
         <f>IF(OR(L20&gt;=척도!$B$17,AND(I20&gt;=척도!$B$19,L20&gt;=척도!$B$18)),"높음",IF(L20&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
@@ -6304,11 +6304,11 @@
       </c>
       <c r="L21" s="11">
         <f>I21*J21*K21</f>
-        <v/>
-      </c>
-      <c r="M21" s="11">
+        <v>252</v>
+      </c>
+      <c r="M21" s="11" t="str">
         <f>IF(OR(L21&gt;=척도!$B$17,AND(I21&gt;=척도!$B$19,L21&gt;=척도!$B$18)),"높음",IF(L21&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
@@ -6523,11 +6523,11 @@
       </c>
       <c r="L5" s="11">
         <f>I5*J5*K5</f>
-        <v/>
-      </c>
-      <c r="M5" s="11">
+        <v>252</v>
+      </c>
+      <c r="M5" s="11" t="str">
         <f>IF(OR(L5&gt;=척도!$B$17,AND(I5&gt;=척도!$B$19,L5&gt;=척도!$B$18)),"높음",IF(L5&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N5" s="12" t="inlineStr">
         <is>
@@ -6590,11 +6590,11 @@
       </c>
       <c r="L6" s="11">
         <f>I6*J6*K6</f>
-        <v/>
-      </c>
-      <c r="M6" s="11">
+        <v>336</v>
+      </c>
+      <c r="M6" s="11" t="str">
         <f>IF(OR(L6&gt;=척도!$B$17,AND(I6&gt;=척도!$B$19,L6&gt;=척도!$B$18)),"높음",IF(L6&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
@@ -6657,11 +6657,11 @@
       </c>
       <c r="L7" s="11">
         <f>I7*J7*K7</f>
-        <v/>
-      </c>
-      <c r="M7" s="11">
+        <v>252</v>
+      </c>
+      <c r="M7" s="11" t="str">
         <f>IF(OR(L7&gt;=척도!$B$17,AND(I7&gt;=척도!$B$19,L7&gt;=척도!$B$18)),"높음",IF(L7&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N7" s="12" t="inlineStr">
         <is>
@@ -6724,11 +6724,11 @@
       </c>
       <c r="L8" s="11">
         <f>I8*J8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="11">
+        <v>336</v>
+      </c>
+      <c r="M8" s="11" t="str">
         <f>IF(OR(L8&gt;=척도!$B$17,AND(I8&gt;=척도!$B$19,L8&gt;=척도!$B$18)),"높음",IF(L8&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
@@ -6791,11 +6791,11 @@
       </c>
       <c r="L9" s="11">
         <f>I9*J9*K9</f>
-        <v/>
-      </c>
-      <c r="M9" s="11">
+        <v>392</v>
+      </c>
+      <c r="M9" s="11" t="str">
         <f>IF(OR(L9&gt;=척도!$B$17,AND(I9&gt;=척도!$B$19,L9&gt;=척도!$B$18)),"높음",IF(L9&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N9" s="12" t="inlineStr">
         <is>
@@ -6858,11 +6858,11 @@
       </c>
       <c r="L10" s="11">
         <f>I10*J10*K10</f>
-        <v/>
-      </c>
-      <c r="M10" s="11">
+        <v>392</v>
+      </c>
+      <c r="M10" s="11" t="str">
         <f>IF(OR(L10&gt;=척도!$B$17,AND(I10&gt;=척도!$B$19,L10&gt;=척도!$B$18)),"높음",IF(L10&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
@@ -6925,11 +6925,11 @@
       </c>
       <c r="L11" s="11">
         <f>I11*J11*K11</f>
-        <v/>
-      </c>
-      <c r="M11" s="11">
+        <v>294</v>
+      </c>
+      <c r="M11" s="11" t="str">
         <f>IF(OR(L11&gt;=척도!$B$17,AND(I11&gt;=척도!$B$19,L11&gt;=척도!$B$18)),"높음",IF(L11&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
@@ -6992,11 +6992,11 @@
       </c>
       <c r="L12" s="11">
         <f>I12*J12*K12</f>
-        <v/>
-      </c>
-      <c r="M12" s="11">
+        <v>72</v>
+      </c>
+      <c r="M12" s="11" t="str">
         <f>IF(OR(L12&gt;=척도!$B$17,AND(I12&gt;=척도!$B$19,L12&gt;=척도!$B$18)),"높음",IF(L12&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>낮음</v>
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
@@ -7059,11 +7059,11 @@
       </c>
       <c r="L13" s="11">
         <f>I13*J13*K13</f>
-        <v/>
-      </c>
-      <c r="M13" s="11">
+        <v>336</v>
+      </c>
+      <c r="M13" s="11" t="str">
         <f>IF(OR(L13&gt;=척도!$B$17,AND(I13&gt;=척도!$B$19,L13&gt;=척도!$B$18)),"높음",IF(L13&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N13" s="12" t="inlineStr">
         <is>
@@ -7126,11 +7126,11 @@
       </c>
       <c r="L14" s="11">
         <f>I14*J14*K14</f>
-        <v/>
-      </c>
-      <c r="M14" s="11">
+        <v>294</v>
+      </c>
+      <c r="M14" s="11" t="str">
         <f>IF(OR(L14&gt;=척도!$B$17,AND(I14&gt;=척도!$B$19,L14&gt;=척도!$B$18)),"높음",IF(L14&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N14" s="12" t="inlineStr">
         <is>
@@ -7193,11 +7193,11 @@
       </c>
       <c r="L15" s="11">
         <f>I15*J15*K15</f>
-        <v/>
-      </c>
-      <c r="M15" s="11">
+        <v>392</v>
+      </c>
+      <c r="M15" s="11" t="str">
         <f>IF(OR(L15&gt;=척도!$B$17,AND(I15&gt;=척도!$B$19,L15&gt;=척도!$B$18)),"높음",IF(L15&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
@@ -7260,11 +7260,11 @@
       </c>
       <c r="L16" s="11">
         <f>I16*J16*K16</f>
-        <v/>
-      </c>
-      <c r="M16" s="11">
+        <v>294</v>
+      </c>
+      <c r="M16" s="11" t="str">
         <f>IF(OR(L16&gt;=척도!$B$17,AND(I16&gt;=척도!$B$19,L16&gt;=척도!$B$18)),"높음",IF(L16&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N16" s="12" t="inlineStr">
         <is>
@@ -7327,11 +7327,11 @@
       </c>
       <c r="L17" s="11">
         <f>I17*J17*K17</f>
-        <v/>
-      </c>
-      <c r="M17" s="11">
+        <v>245</v>
+      </c>
+      <c r="M17" s="11" t="str">
         <f>IF(OR(L17&gt;=척도!$B$17,AND(I17&gt;=척도!$B$19,L17&gt;=척도!$B$18)),"높음",IF(L17&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N17" s="12" t="inlineStr">
         <is>
@@ -7394,11 +7394,11 @@
       </c>
       <c r="L18" s="11">
         <f>I18*J18*K18</f>
-        <v/>
-      </c>
-      <c r="M18" s="11">
+        <v>343</v>
+      </c>
+      <c r="M18" s="11" t="str">
         <f>IF(OR(L18&gt;=척도!$B$17,AND(I18&gt;=척도!$B$19,L18&gt;=척도!$B$18)),"높음",IF(L18&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
@@ -7461,11 +7461,11 @@
       </c>
       <c r="L19" s="11">
         <f>I19*J19*K19</f>
-        <v/>
-      </c>
-      <c r="M19" s="11">
+        <v>392</v>
+      </c>
+      <c r="M19" s="11" t="str">
         <f>IF(OR(L19&gt;=척도!$B$17,AND(I19&gt;=척도!$B$19,L19&gt;=척도!$B$18)),"높음",IF(L19&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
@@ -7528,11 +7528,11 @@
       </c>
       <c r="L20" s="11">
         <f>I20*J20*K20</f>
-        <v/>
-      </c>
-      <c r="M20" s="11">
+        <v>294</v>
+      </c>
+      <c r="M20" s="11" t="str">
         <f>IF(OR(L20&gt;=척도!$B$17,AND(I20&gt;=척도!$B$19,L20&gt;=척도!$B$18)),"높음",IF(L20&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>중간</v>
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
@@ -7595,11 +7595,11 @@
       </c>
       <c r="L21" s="11">
         <f>I21*J21*K21</f>
-        <v/>
-      </c>
-      <c r="M21" s="11">
+        <v>378</v>
+      </c>
+      <c r="M21" s="11" t="str">
         <f>IF(OR(L21&gt;=척도!$B$17,AND(I21&gt;=척도!$B$19,L21&gt;=척도!$B$18)),"높음",IF(L21&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
@@ -7662,11 +7662,11 @@
       </c>
       <c r="L22" s="11">
         <f>I22*J22*K22</f>
-        <v/>
-      </c>
-      <c r="M22" s="11">
+        <v>336</v>
+      </c>
+      <c r="M22" s="11" t="str">
         <f>IF(OR(L22&gt;=척도!$B$17,AND(I22&gt;=척도!$B$19,L22&gt;=척도!$B$18)),"높음",IF(L22&gt;=척도!$B$18,"중간","낮음"))</f>
-        <v/>
+        <v>높음</v>
       </c>
       <c r="N22" s="12" t="inlineStr">
         <is>
@@ -7770,27 +7770,27 @@
       </c>
       <c r="B4" s="9">
         <f>COUNTA('FMEA_일반'!A5:A63)</f>
-        <v/>
+        <v>59</v>
       </c>
       <c r="C4" s="9">
         <f>COUNTIF('FMEA_일반'!M5:M63,"높음")</f>
-        <v/>
+        <v>17</v>
       </c>
       <c r="D4" s="9">
         <f>COUNTIF('FMEA_일반'!M5:M63,"중간")</f>
-        <v/>
+        <v>35</v>
       </c>
       <c r="E4" s="9">
         <f>COUNTIF('FMEA_일반'!M5:M63,"낮음")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="F4" s="14">
         <f>AVERAGE('FMEA_일반'!L5:L63)</f>
-        <v/>
+        <v>252.83050847457628</v>
       </c>
       <c r="G4" s="9">
         <f>MAX('FMEA_일반'!L5:L63)</f>
-        <v/>
+        <v>378</v>
       </c>
     </row>
     <row r="5">
@@ -7801,27 +7801,27 @@
       </c>
       <c r="B5" s="9">
         <f>COUNTA('FMEA_교육자격'!A5:A21)</f>
-        <v/>
+        <v>17</v>
       </c>
       <c r="C5" s="9">
         <f>COUNTIF('FMEA_교육자격'!M5:M21,"높음")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="D5" s="9">
         <f>COUNTIF('FMEA_교육자격'!M5:M21,"중간")</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="E5" s="9">
         <f>COUNTIF('FMEA_교육자격'!M5:M21,"낮음")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F5" s="14">
         <f>AVERAGE('FMEA_교육자격'!L5:L21)</f>
-        <v/>
+        <v>301.88235294117646</v>
       </c>
       <c r="G5" s="9">
         <f>MAX('FMEA_교육자격'!L5:L21)</f>
-        <v/>
+        <v>441</v>
       </c>
     </row>
     <row r="6">
@@ -7832,27 +7832,27 @@
       </c>
       <c r="B6" s="9">
         <f>COUNTA('FMEA_모의훈련'!A5:A22)</f>
-        <v/>
+        <v>18</v>
       </c>
       <c r="C6" s="9">
         <f>COUNTIF('FMEA_모의훈련'!M5:M22,"높음")</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="D6" s="9">
         <f>COUNTIF('FMEA_모의훈련'!M5:M22,"중간")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="E6" s="9">
         <f>COUNTIF('FMEA_모의훈련'!M5:M22,"낮음")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F6" s="14">
         <f>AVERAGE('FMEA_모의훈련'!L5:L22)</f>
-        <v/>
+        <v>312.77777777777777</v>
       </c>
       <c r="G6" s="9">
         <f>MAX('FMEA_모의훈련'!L5:L22)</f>
-        <v/>
+        <v>392</v>
       </c>
     </row>
     <row r="7">
@@ -7863,19 +7863,19 @@
       </c>
       <c r="B7" s="11">
         <f>SUM(B4:B6)</f>
-        <v/>
+        <v>94</v>
       </c>
       <c r="C7" s="11">
         <f>SUM(C4:C6)</f>
-        <v/>
+        <v>33</v>
       </c>
       <c r="D7" s="11">
         <f>SUM(D4:D6)</f>
-        <v/>
+        <v>53</v>
       </c>
       <c r="E7" s="11">
         <f>SUM(E4:E6)</f>
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -7915,15 +7915,15 @@
       </c>
       <c r="B11" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A11)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C11" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A11,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>238.0</v>
       </c>
       <c r="D11" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A11,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -7934,15 +7934,15 @@
       </c>
       <c r="B12" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A12)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="C12" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A12,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>264.0</v>
       </c>
       <c r="D12" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A12,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -7953,15 +7953,15 @@
       </c>
       <c r="B13" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A13)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C13" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A13,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>223.33333333333334</v>
       </c>
       <c r="D13" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A13,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -7972,15 +7972,15 @@
       </c>
       <c r="B14" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A14)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="C14" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A14,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>263.4</v>
       </c>
       <c r="D14" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A14,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -7991,15 +7991,15 @@
       </c>
       <c r="B15" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A15)</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="C15" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A15,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>256.7692307692308</v>
       </c>
       <c r="D15" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A15,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -8010,15 +8010,15 @@
       </c>
       <c r="B16" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A16)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="C16" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A16,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>226.57142857142858</v>
       </c>
       <c r="D16" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A16,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -8029,15 +8029,15 @@
       </c>
       <c r="B17" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A17)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="C17" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A17,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>244.8</v>
       </c>
       <c r="D17" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A17,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -8048,15 +8048,15 @@
       </c>
       <c r="B18" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A18)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C18" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A18,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>272.0</v>
       </c>
       <c r="D18" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A18,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -8067,15 +8067,15 @@
       </c>
       <c r="B19" s="9">
         <f>COUNTIF('FMEA_일반'!$B$5:$B$63,A19)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C19" s="14">
         <f>AVERAGEIF('FMEA_일반'!$B$5:$B$63,A19,'FMEA_일반'!$L$5:$L$63)</f>
-        <v/>
+        <v>339.5</v>
       </c>
       <c r="D19" s="9">
         <f>COUNTIFS('FMEA_일반'!$B$5:$B$63,A19,'FMEA_일반'!$M$5:$M$63,"높음")</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -8110,11 +8110,11 @@
       </c>
       <c r="B23" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A23)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C23" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A23,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>291.0</v>
       </c>
     </row>
     <row r="24">
@@ -8125,11 +8125,11 @@
       </c>
       <c r="B24" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A24)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C24" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A24,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>240.0</v>
       </c>
     </row>
     <row r="25">
@@ -8140,11 +8140,11 @@
       </c>
       <c r="B25" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A25)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C25" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A25,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>343.0</v>
       </c>
     </row>
     <row r="26">
@@ -8155,11 +8155,11 @@
       </c>
       <c r="B26" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A26)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="C26" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A26,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>269.3333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -8170,11 +8170,11 @@
       </c>
       <c r="B27" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A27)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="C27" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A27,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>347.6666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -8185,11 +8185,11 @@
       </c>
       <c r="B28" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A28)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="C28" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A28,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>315.0</v>
       </c>
     </row>
     <row r="29">
@@ -8200,11 +8200,11 @@
       </c>
       <c r="B29" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A29)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C29" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A29,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>294.0</v>
       </c>
     </row>
     <row r="30">
@@ -8215,11 +8215,11 @@
       </c>
       <c r="B30" s="9">
         <f>COUNTIF('FMEA_교육자격'!$D$5:$D$21,A30)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C30" s="14">
         <f>AVERAGEIF('FMEA_교육자격'!$D$5:$D$21,A30,'FMEA_교육자격'!$L$5:$L$21)</f>
-        <v/>
+        <v>315.0</v>
       </c>
     </row>
     <row r="32">
@@ -8254,11 +8254,11 @@
       </c>
       <c r="B34" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A34)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C34" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A34,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>294.0</v>
       </c>
     </row>
     <row r="35">
@@ -8269,11 +8269,11 @@
       </c>
       <c r="B35" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A35)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C35" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A35,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>294.0</v>
       </c>
     </row>
     <row r="36">
@@ -8284,11 +8284,11 @@
       </c>
       <c r="B36" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A36)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="C36" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A36,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>287.5</v>
       </c>
     </row>
     <row r="37">
@@ -8299,11 +8299,11 @@
       </c>
       <c r="B37" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A37)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C37" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A37,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>315.0</v>
       </c>
     </row>
     <row r="38">
@@ -8314,11 +8314,11 @@
       </c>
       <c r="B38" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A38)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="C38" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A38,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>310.3333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -8329,11 +8329,11 @@
       </c>
       <c r="B39" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A39)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="C39" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A39,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>343.0</v>
       </c>
     </row>
     <row r="40">
@@ -8344,11 +8344,11 @@
       </c>
       <c r="B40" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A40)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C40" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A40,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>343.0</v>
       </c>
     </row>
     <row r="41">
@@ -8359,11 +8359,11 @@
       </c>
       <c r="B41" s="9">
         <f>COUNTIF('FMEA_모의훈련'!$D$5:$D$22,A41)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C41" s="14">
         <f>AVERAGEIF('FMEA_모의훈련'!$D$5:$D$22,A41,'FMEA_모의훈련'!$L$5:$L$22)</f>
-        <v/>
+        <v>357.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>